<commit_message>
Add some more details from the amisulbrom DAR
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/amisulbrom_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/amisulbrom_aquatic_toxicity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B4AD80-4D28-4E21-8D4E-DEA008F60837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F48FB2-0AFA-4131-9AB2-2CA44028F118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DCCE98E3-7ECB-464D-B3A9-333AAEFCC845}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="70">
   <si>
     <t>substance</t>
   </si>
@@ -201,9 +201,6 @@
     <t>Equivalent to 0.25 mg formulation/L</t>
   </si>
   <si>
-    <t>Effect not specified in table; NOEC reported</t>
-  </si>
-  <si>
     <t>Equivalent to 0.24 mg formulation/L</t>
   </si>
   <si>
@@ -241,6 +238,15 @@
   </si>
   <si>
     <t>rajo</t>
+  </si>
+  <si>
+    <t>Measured concentrations are not further specified in the RAR, so it is not clear if they are geometric mean measured or e.g. initial measured.</t>
+  </si>
+  <si>
+    <t>early life stage</t>
+  </si>
+  <si>
+    <t>Effect not specified in table; NOEC reported; measured concentrations seem to be initial measured</t>
   </si>
 </sst>
 </file>
@@ -713,11 +719,11 @@
     </row>
     <row r="2" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -745,41 +751,41 @@
         <v>26</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>57</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>57</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>65</v>
       </c>
       <c r="S2" s="3">
         <v>611</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V2" s="3"/>
       <c r="W2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X2" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X2" s="5" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="3" spans="1:24" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D3" s="3">
         <v>2</v>
@@ -806,36 +812,42 @@
       <c r="N3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="3"/>
+      <c r="O3" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P3" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q3" s="3">
         <v>57</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S3" s="3">
+        <v>613</v>
+      </c>
       <c r="T3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V3" s="3"/>
       <c r="W3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X3" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D4" s="3">
         <v>3</v>
@@ -862,32 +874,38 @@
       <c r="N4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="3"/>
+      <c r="O4" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P4" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q4" s="3">
         <v>57</v>
       </c>
-      <c r="R4"/>
-      <c r="S4"/>
+      <c r="R4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S4">
+        <v>615</v>
+      </c>
       <c r="T4" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V4"/>
       <c r="W4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X4" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
@@ -918,32 +936,38 @@
       <c r="N5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O5" s="3"/>
+      <c r="O5" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P5" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q5" s="2">
         <v>58</v>
       </c>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
+      <c r="R5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S5" s="3">
+        <v>617</v>
+      </c>
       <c r="T5" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V5" s="3"/>
       <c r="W5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X5" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X5" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
@@ -974,32 +998,38 @@
       <c r="N6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="3"/>
+      <c r="O6" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P6" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q6" s="2">
         <v>58</v>
       </c>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
+      <c r="R6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S6" s="3">
+        <v>619</v>
+      </c>
       <c r="T6" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U6" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V6" s="3"/>
       <c r="W6" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X6" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X6" s="5" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3" t="s">
@@ -1032,30 +1062,36 @@
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q7" s="2">
         <v>58</v>
       </c>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
+      <c r="R7" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S7" s="3">
+        <v>621</v>
+      </c>
       <c r="T7" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U7" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="V7" s="3"/>
+        <v>58</v>
+      </c>
+      <c r="V7" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="W7" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X7" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X7" s="5" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3" t="s">
@@ -1071,7 +1107,9 @@
       <c r="G8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="3"/>
+      <c r="H8" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="I8" s="3" t="s">
         <v>27</v>
       </c>
@@ -1088,30 +1126,36 @@
       </c>
       <c r="O8" s="3"/>
       <c r="P8" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q8" s="2">
         <v>58</v>
       </c>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
+      <c r="R8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S8" s="3">
+        <v>645</v>
+      </c>
       <c r="T8" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="V8" s="3"/>
+        <v>58</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="W8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X8" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X8" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>49</v>
@@ -1144,33 +1188,40 @@
       <c r="N9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O9" s="3"/>
+      <c r="O9" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P9" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q9" s="2">
         <v>58</v>
       </c>
-      <c r="S9" s="3"/>
+      <c r="R9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S9" s="3">
+        <v>619</v>
+      </c>
       <c r="T9" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U9" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V9" s="3" t="s">
         <v>50</v>
       </c>
       <c r="W9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X9" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X9" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
@@ -1201,31 +1252,38 @@
       <c r="N10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O10" s="3"/>
+      <c r="O10" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P10" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q10" s="2">
         <v>58</v>
       </c>
-      <c r="S10" s="3"/>
+      <c r="R10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S10" s="3">
+        <v>623</v>
+      </c>
       <c r="T10" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U10" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V10" s="3"/>
       <c r="W10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X10" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X10" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3" t="s">
@@ -1258,33 +1316,40 @@
       <c r="N11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O11" s="3"/>
+      <c r="O11" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P11" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q11" s="2">
         <v>58</v>
       </c>
-      <c r="S11" s="3"/>
+      <c r="R11" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S11" s="3">
+        <v>648</v>
+      </c>
       <c r="T11" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U11" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V11" s="3" t="s">
         <v>52</v>
       </c>
       <c r="W11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X11" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X11" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>49</v>
@@ -1317,33 +1382,40 @@
       <c r="N12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O12" s="3"/>
+      <c r="O12" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P12" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q12" s="2">
         <v>58</v>
       </c>
-      <c r="S12" s="3"/>
+      <c r="R12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S12" s="3">
+        <v>641</v>
+      </c>
       <c r="T12" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U12" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V12" s="3" t="s">
         <v>53</v>
       </c>
       <c r="W12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X12" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X12" s="5" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="13" spans="1:24" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
@@ -1374,31 +1446,36 @@
       </c>
       <c r="O13" s="3"/>
       <c r="P13" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q13" s="2">
         <v>58</v>
       </c>
-      <c r="S13" s="3"/>
+      <c r="R13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S13" s="3">
+        <v>655</v>
+      </c>
       <c r="T13" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U13" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V13" s="3" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="W13" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X13" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X13" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3" t="s">
@@ -1429,33 +1506,40 @@
       <c r="N14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O14" s="3"/>
+      <c r="O14" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P14" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q14" s="2">
         <v>58</v>
       </c>
-      <c r="S14" s="3"/>
+      <c r="R14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S14" s="3">
+        <v>625</v>
+      </c>
       <c r="T14" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U14" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V14" s="3" t="s">
         <v>46</v>
       </c>
       <c r="W14" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X14" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X14" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3" t="s">
@@ -1486,33 +1570,40 @@
       <c r="N15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O15" s="3"/>
+      <c r="O15" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P15" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q15" s="2">
         <v>58</v>
       </c>
-      <c r="S15" s="3"/>
+      <c r="R15" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S15" s="3">
+        <v>625</v>
+      </c>
       <c r="T15" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U15" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V15" s="3" t="s">
         <v>40</v>
       </c>
       <c r="W15" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X15" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X15" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>49</v>
@@ -1545,33 +1636,40 @@
       <c r="N16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O16" s="3"/>
+      <c r="O16" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P16" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q16" s="2">
         <v>58</v>
       </c>
-      <c r="S16" s="3"/>
+      <c r="R16" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S16" s="3">
+        <v>642</v>
+      </c>
       <c r="T16" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U16" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="W16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X16" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X16" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>49</v>
@@ -1604,28 +1702,35 @@
       <c r="N17" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O17" s="3"/>
+      <c r="O17" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="P17" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q17" s="2">
         <v>58</v>
       </c>
-      <c r="S17" s="3"/>
+      <c r="R17" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S17" s="3">
+        <v>642</v>
+      </c>
       <c r="T17" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U17" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V17" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="W17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X17" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="X17" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>